<commit_message>
Se integró la HU05 y la HU07.Falta darle formato de tarjeta, Paolo.
</commit_message>
<xml_diff>
--- a/docs/Historias de usuario/Tabla de HU.xlsx
+++ b/docs/Historias de usuario/Tabla de HU.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\utp7\Diseño de Productos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\utp7\Diseño de Productos\EcoSolido\docs\Historias de usuario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EF2F647-DCAF-4CEE-BC5D-E38329321B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4CFBD9-B645-4775-86F0-39BCD6CCC982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0DA53D5F-3327-48A2-BB14-3877498098E0}"/>
   </bookViews>
@@ -164,20 +164,6 @@
     <t>Módulo de Registro de Incidencias</t>
   </si>
   <si>
-    <t>Escenario 1: Ciudadano registra una incidencia con fotos y descripción
-GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
-WHEN: El ciudadano adjunta al menos 1 foto e ingresa una descripción del problema.
-THEN: El sistema guarda la incidencia, muestra "Tu incidencia ha sido registrada exitosamente" y le asigna el estado "Pendiente".
-Escenario 2: Ciudadano intenta registrar sin descripción
-GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
-WHEN: El ciudadano adjunta fotos pero no ingresa descripción y presiona registrar.
-THEN: El sistema muestra un mensaje de error indicando que la descripción es obligatoria.
-Escenario 3: Ciudadano intenta registrar sin fotos
-GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
-WHEN: El ciudadano ingresa una descripción pero no adjunta ninguna foto y presiona registrar.
-THEN: El sistema muestra un mensaje de error indicando que debe adjuntar al menos una foto.</t>
-  </si>
-  <si>
     <t>Escenario 1: Ciudadano usa GPS para establecer su ubicación
 GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
 WHEN: El ciudadano presiona "Usar mi ubicación actual" y acepta el permiso de GPS.
@@ -350,6 +336,36 @@
 GIVEN:El sistema mostró la pregunta de seguridad
 WHEN:El ciudadano responde correctamente
 THEN:La aplicación habilita el formulario para ingresar y confirmar una nueva contraseña.</t>
+  </si>
+  <si>
+    <t>Escenario 1: Ciudadano registra una incidencia con fotos y descripción
+GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
+WHEN: El ciudadano adjunta al menos 1 foto , ingresa una descripción de la incidencia y la categoría relacionada a la incidencia.
+THEN: El sistema guarda la incidencia, muestra "Tu incidencia ha sido registrada exitosamente" y le asigna el estado "Pendiente".
+Escenario 2: Ciudadano quiere generar una descripción usando las fotos
+GIVEN: El ciudadano ha adjuntado fotos para registrar la incidencia y ha presionado en el botón “Generar descripción por IA.
+WHEN: El ciudadano confirma que quiere generar la descripción en base a las fotos.
+THEN: El sistema genera texto en el cuadro de texto relacionado a la descripción de la incidencia en base a las fotos usando la API de Hugging Face.
+Escenario 3: La IA de Hugging Face no puede describir correctamente la foto
+GIVEN: El ciudadano ha adjuntado fotos para registrar la incidencia y ha presionado en el botón “Generar descripción por IA.
+WHEN: El ciudadano confirma que quiere generar la descripción en base a las fotos.
+THEN: El sistema genera un texto dentro del cuadro el cuál dice: “No se ha podido describir la foto”.
+Escenario 4: El ciudadano deniega hacer el texto con IA 
+GIVEN: El ciudadano ha adjuntado fotos para registrar la incidencia y ha presionado en el botón “Generar descripción por IA.
+WHEN: El ciudadano no acepta que quiere generar la descripción en base a las fotos.
+THEN: La ventana flotante desaparece y no se agrega texto.
+Escenario 5: Ciudadano intenta registrar incidencia  sin descripción
+GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
+WHEN: El ciudadano adjunta fotos, establece la categoría pero no ingresa descripción y presiona registrar.
+THEN: El sistema muestra un mensaje de error indicando que la descripción es obligatoria.
+Escenario 6: Ciudadano intenta registrar incidencia sin fotos
+GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
+WHEN: El ciudadano ingresa una descripción, establece la categoría pero no adjunta ninguna foto y presiona registrar.
+THEN: El sistema muestra un mensaje de error indicando que debe adjuntar al menos una foto.
+Escenario 7: Ciudadano intenta registrar una incidencia sin establecer su categoría
+GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
+WHEN: El ciudadano ingresa una descripción y adjunta fotos pero no establece la categoría de la incidencia.
+THEN: El sistema muestra un mensaje de error indicando que debe establecer la categoría de la incidencia..</t>
   </si>
 </sst>
 </file>
@@ -917,7 +933,7 @@
   <sheetData>
     <row r="3" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="10"/>
@@ -948,7 +964,7 @@
         <v>12</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="192.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -969,10 +985,10 @@
         <v>7</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="183" customHeight="1" x14ac:dyDescent="0.3">
@@ -981,15 +997,15 @@
         <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="228.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>9</v>
@@ -1007,7 +1023,7 @@
         <v>10</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>26</v>
@@ -1019,15 +1035,15 @@
         <v>11</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="201.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>16</v>
@@ -1045,24 +1061,24 @@
         <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="240.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>19</v>
       </c>
       <c r="C14" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="336" customHeight="1" x14ac:dyDescent="0.3">
@@ -1071,10 +1087,10 @@
         <v>20</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="364.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1083,10 +1099,10 @@
         <v>21</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="331.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1095,13 +1111,13 @@
         <v>22</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="345.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="409.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>29</v>
       </c>
@@ -1109,10 +1125,10 @@
         <v>23</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="349.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1124,7 +1140,7 @@
         <v>25</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Nuevo escenario para el módulo de Seguimiento de incidencia
</commit_message>
<xml_diff>
--- a/docs/Historias de usuario/Tabla de HU.xlsx
+++ b/docs/Historias de usuario/Tabla de HU.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\utp7\Diseño de Productos\EcoSolido\docs\Historias de usuario\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\utp7\Diseño de Productos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4CFBD9-B645-4775-86F0-39BCD6CCC982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F263D032-73B4-4193-A069-75A85286CD1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0DA53D5F-3327-48A2-BB14-3877498098E0}"/>
   </bookViews>
@@ -83,16 +83,6 @@
 para registrar una incidencia en el menor tiempo posible.</t>
   </si>
   <si>
-    <t>Escenario 1: Ciudadano inicia sesión correctamente
-GIVEN: El ciudadano ingresa su nombre de usuario y contraseña.
-WHEN: El ciudadano presiona el botón Ingresar.
-THEN: El ciudadano es redirigido al panel de registrar incidencia con la barra de navegación al lado.
-Escenario 2: Ciudadano ingresa credenciales incorrectas
-GIVEN: El ciudadano ingresa un nombre de usuario o contraseña incorrectos.
-WHEN: El conductor presiona el botón "Ingresar".
-THEN: La aplicación muestra un mensaje de error indicando que las credenciales son incorrectas.</t>
-  </si>
-  <si>
     <t>Como ciudadano,
 necesito visualizar métricas de mis incidencias reportadas 
 para comprobar que realmente estoy contribuyendo a la gestión de residuos en mi distrito.</t>
@@ -129,26 +119,6 @@
   <si>
     <t>Como ciudadano, necesito indicar la ubicación exacta del problema 
 para que el equipo de recolección pueda encontrar la ruta más óptima y lleguen en el menor tiempo posible.</t>
-  </si>
-  <si>
-    <t>Escenario 1: Ciudadano consulta el estado de su reporte
-GIVEN: El ciudadano ha iniciado sesión correctamente.
-WHEN: El ciudadano presiona "Seguimiento de Incidencias reportadas" en la barra de navegación.
-THEN: La aplicación muestra una lista de reportes con fecha, descripción breve y estado actual (Pendiente, En Proceso o Resuelto).
-Escenario 2: Ciudadano no tiene reportes registrados
-GIVEN: El ciudadano ha iniciado sesión y no ha creado ningún reporte.
-WHEN: El ciudadano presiona " Seguimiento de Incidencias reportadas".
-THEN: La aplicación muestra un mensaje indicando que aún no tiene reportes registrados.</t>
-  </si>
-  <si>
-    <t>Escenario 1: Ciudadano visualiza sus métricas personales
-GIVEN: El ciudadano ha iniciado sesión en la aplicación.
-WHEN: El ciudadano presiona "Seguimiento de Incidencias Registradas" en la barra de navegación.
-THEN: El sistema muestra un panel con: total de incidencias reportadas, total resueltas y total en proceso.
-Escenario 2: Ciudadano aún no tiene incidencias registradas
-GIVEN: El ciudadano ha iniciado sesión y no ha reportado ninguna incidencia.
-WHEN: El ciudadano presiona "Seguimiento de incidencias registradas".
-THEN: El sistema muestra el panel con métricas en cero y el mensaje: "¡Empieza a reportar incidencias y mide tu impacto!"</t>
   </si>
   <si>
     <t>Escenario 1: Ciudadano accede a noticias medioambientales
@@ -162,6 +132,20 @@
   </si>
   <si>
     <t>Módulo de Registro de Incidencias</t>
+  </si>
+  <si>
+    <t>Escenario 1: Ciudadano registra una incidencia con fotos y descripción
+GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
+WHEN: El ciudadano adjunta al menos 1 foto e ingresa una descripción del problema.
+THEN: El sistema guarda la incidencia, muestra "Tu incidencia ha sido registrada exitosamente" y le asigna el estado "Pendiente".
+Escenario 2: Ciudadano intenta registrar sin descripción
+GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
+WHEN: El ciudadano adjunta fotos pero no ingresa descripción y presiona registrar.
+THEN: El sistema muestra un mensaje de error indicando que la descripción es obligatoria.
+Escenario 3: Ciudadano intenta registrar sin fotos
+GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
+WHEN: El ciudadano ingresa una descripción pero no adjunta ninguna foto y presiona registrar.
+THEN: El sistema muestra un mensaje de error indicando que debe adjuntar al menos una foto.</t>
   </si>
   <si>
     <t>Escenario 1: Ciudadano usa GPS para establecer su ubicación
@@ -221,16 +205,6 @@
  para mantener mi vecindario limpio.</t>
   </si>
   <si>
-    <t>Escenario 1: Ciudadano consulta consejos sobre un tipo de residuo
-GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Educación Medioambiental".
-WHEN: El ciudadano selecciona "Residuos Orgánicos" en el combobox y confirma la consulta.
-THEN: La aplicación muestra al menos 2 recomendaciones que contribuyen al manejo correcto de ese tipo de residuo.
-Escenario 2: Ciudadano no selecciona ningún tipo de residuo
-GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Educación Medioambiental".
-WHEN: El ciudadano intenta consultar sin seleccionar un tipo de residuo.
-THEN: El sistema muestra un mensaje solicitando que seleccione un tipo de residuo antes de continuar.</t>
-  </si>
-  <si>
     <t>Como ciudadano, quiero ver cuántos puntos he acumulado por mis incidencias registradas para saber cuánto he contribuido al distrito.</t>
   </si>
   <si>
@@ -242,20 +216,6 @@
 GIVEN: El ciudadano ha iniciado sesión pero no ha registrado ninguna incidencia
 WHEN:Accede a la sección "Mis puntos" dentro del módulo de recompensas al ciudadano
 THEN: El sistema muestra 0 puntos e indica que aún no ha realizado contribuciones</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Escenario 1: El sistema asigna puntos tras un registro exitoso
-GIVEN: El ciudadano ha completado y enviado correctamente una incidencia según HU014
-WHEN: El sistema confirma el registro de la incidencia
-THEN: El sistema asigna automáticamente los puntos correspondientes y notifica al ciudadano la cantidad de puntos ganados
-Escenario 2: Los puntos se reflejan inmediatamente en el perfil del ciudadano
-GIVEN:El ciudadano acaba de registrar una incidencia y el sistema le asignó puntos
-WHEN:El ciudadano accede a su perfil o sección "Mis puntos"
-THEN:El total de puntos mostrado incluye los puntos recién ganados
-Escenario 3:Incidencia duplicada no genera puntos adicionales
-GIVEN: El ciudadano intenta registrar una incidencia idéntica a una ya reportada por él
-WHEN: El sistema detecta la duplicidad y rechaza el registro
-THEN: No se asignan puntos adicionales y el sistema notifica que la incidencia ya fue registrada</t>
   </si>
   <si>
     <t>Escenario 1: Ciudadano visualiza el ranking general
@@ -300,20 +260,6 @@
 THEN: La aplicación no muestra ningún reporte con el mensaje de no hay ningún reporte de tal tipo.</t>
   </si>
   <si>
-    <t>Escenario 1: Ciudadano se crea una cuenta
-GIVEN:El ciudadano completa todos los campos: nombre completo, DNI, nombre de usuario, contraseña, confirmación de contraseña y pregunta de seguridad
-WHEN:El ciudadano presiona el botón "Crear cuenta"
-THEN:El sistema registra la cuenta y redirige al ciudadano al inicio de sesión
-Escenario 2: Las contraseñas no coinciden
-GIVEN:El ciudadano completa el formulario pero ingresa una confirmación de contraseña diferente
-WHEN:El ciudadano presiona "Crear cuenta"
-THEN:El sistema muestra un mensaje indicando que las contraseñas no coinciden y no crea la cuenta
-Escenario 3: Campos obligatorios vacíos
-GIVEN:El ciudadano deja uno o más campos sin completar
-WHEN:El ciudadano presiona "Crear cuenta"
-THEN:El sistema resalta los campos vacíos e indica que son obligatorios</t>
-  </si>
-  <si>
     <t>Escenario 1: El ciudadano confirma que quiere cerrar sesión
 GIVEN: El ciudadano presionó el botón cerrar sesión.
 WHEN: El ciudadano confirmó la acción presionando "cerrar sesión" en la ventana de confirmación.
@@ -338,34 +284,89 @@
 THEN:La aplicación habilita el formulario para ingresar y confirmar una nueva contraseña.</t>
   </si>
   <si>
-    <t>Escenario 1: Ciudadano registra una incidencia con fotos y descripción
-GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
-WHEN: El ciudadano adjunta al menos 1 foto , ingresa una descripción de la incidencia y la categoría relacionada a la incidencia.
-THEN: El sistema guarda la incidencia, muestra "Tu incidencia ha sido registrada exitosamente" y le asigna el estado "Pendiente".
-Escenario 2: Ciudadano quiere generar una descripción usando las fotos
-GIVEN: El ciudadano ha adjuntado fotos para registrar la incidencia y ha presionado en el botón “Generar descripción por IA.
-WHEN: El ciudadano confirma que quiere generar la descripción en base a las fotos.
-THEN: El sistema genera texto en el cuadro de texto relacionado a la descripción de la incidencia en base a las fotos usando la API de Hugging Face.
-Escenario 3: La IA de Hugging Face no puede describir correctamente la foto
-GIVEN: El ciudadano ha adjuntado fotos para registrar la incidencia y ha presionado en el botón “Generar descripción por IA.
-WHEN: El ciudadano confirma que quiere generar la descripción en base a las fotos.
-THEN: El sistema genera un texto dentro del cuadro el cuál dice: “No se ha podido describir la foto”.
-Escenario 4: El ciudadano deniega hacer el texto con IA 
-GIVEN: El ciudadano ha adjuntado fotos para registrar la incidencia y ha presionado en el botón “Generar descripción por IA.
-WHEN: El ciudadano no acepta que quiere generar la descripción en base a las fotos.
-THEN: La ventana flotante desaparece y no se agrega texto.
-Escenario 5: Ciudadano intenta registrar incidencia  sin descripción
-GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
-WHEN: El ciudadano adjunta fotos, establece la categoría pero no ingresa descripción y presiona registrar.
-THEN: El sistema muestra un mensaje de error indicando que la descripción es obligatoria.
-Escenario 6: Ciudadano intenta registrar incidencia sin fotos
-GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
-WHEN: El ciudadano ingresa una descripción, establece la categoría pero no adjunta ninguna foto y presiona registrar.
-THEN: El sistema muestra un mensaje de error indicando que debe adjuntar al menos una foto.
-Escenario 7: Ciudadano intenta registrar una incidencia sin establecer su categoría
-GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Registrar Incidencias".
-WHEN: El ciudadano ingresa una descripción y adjunta fotos pero no establece la categoría de la incidencia.
-THEN: El sistema muestra un mensaje de error indicando que debe establecer la categoría de la incidencia..</t>
+    <t>Escenario 1: Ciudadano inicia sesión correctamente
+GIVEN: El ciudadano ingresa su nombre de usuario y contraseña.
+WHEN: El ciudadano presiona el botón Ingresar.
+THEN: El ciudadano es redirigido al panel de registrar incidencia con la barra de navegación al lado.
+Escenario 2: Ciudadano ingresa credenciales incorrectas
+GIVEN: El ciudadano ingresa un nombre de usuario o contraseña incorrectos.
+WHEN: El ciudadano  presiona el botón "Ingresar".
+THEN: La aplicación muestra un mensaje de error que indica que las credenciales ingresadas son incorrectas. 
+Escenario 3: El servidor se encuentra fuera de servicio
+GIVEN:  El ciudadano ingresa su nombre de usuario y contraseña correctos pero el servidor no está disponible.
+WHEN: El ciudadano presiona el botón Ingresar
+THEN: El ciudadano recibe un mensaje flotante que dice error en el servidor y que vuelva a ingresar más tarde.</t>
+  </si>
+  <si>
+    <t>Escenario 1: Ciudadano se crea una cuenta
+GIVEN:El ciudadano completa todos los campos: nombres y apellidos completos, DNI que este asociado con los nombres y apellidos colocados de acuerdo a la RENIEC, nombre de usuario, contraseña, confirmación de contraseña y pregunta de seguridad
+WHEN:El ciudadano presiona el botón "Crear cuenta"
+THEN:El sistema registra la cuenta y redirige al ciudadano al inicio de sesión
+Escenario 2: Las contraseñas no coinciden
+GIVEN:El ciudadano completa el formulario pero ingresa una confirmación de contraseña diferente
+WHEN:El ciudadano presiona "Crear cuenta"
+THEN:El sistema muestra un mensaje indicando que las contraseñas no coinciden y no crea la cuenta
+Escenario 3: Los nombres no coinciden con el DNI 
+GIVEN:El ciudadano ingresa sus nombres y apellidos correctos pero el DNI no.
+WHEN:El ciudadano presiona "Crear cuenta"
+THEN:El sistema muestra un mensaje el cuál dice que el DNI no coincide con los nombres y apellidos asociados a este en RENIEC.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escenario 1: Ciudadano visualiza sus métricas personales
+GIVEN: El ciudadano ha iniciado sesión en la aplicación.
+WHEN: El ciudadano presiona "Seguimiento de Incidencias Registradas" en la barra de navegación.
+THEN: El sistema muestra un panel con: total de incidencias reportadas, total resueltas y total en proceso.
+Escenario 2: Ciudadano aún no tiene incidencias registradas
+GIVEN: El ciudadano ha iniciado sesión y no ha reportado ninguna incidencia.
+WHEN: El ciudadano presiona "Seguimiento de incidencias registradas".
+THEN: El sistema muestra el panel con métricas en cero y el mensaje: "¡Empieza a reportar incidencias y mide tu impacto!"
+Escenario 3: Ciudadano visualiza métricas actualizadas tras registrar una nueva incidencia
+GIVEN: El ciudadano ha iniciado sesión, tiene incidencias previamente registradas y acaba de registrar una nueva.
+WHEN: El ciudadano presiona "Seguimiento de Incidencias Registradas" en la barra de navegación.
+THEN: El sistema muestra el panel con las métricas actualizadas reflejando la nueva incidencia registrada en el total reportadas.
+</t>
+  </si>
+  <si>
+    <t>Escenario 1: Ciudadano consulta el estado de su reporte
+GIVEN: El ciudadano ha iniciado sesión correctamente.
+WHEN: El ciudadano presiona "Seguimiento de Incidencias reportadas" en la barra de navegación.
+THEN: La aplicación muestra una lista de reportes con fecha, descripción breve, estado actual (Pendiente, En Proceso o Resuelto) y 1 imagen relacionada a la incidencia
+Escenario 2: Ciudadano no tiene reportes registrados
+GIVEN: El ciudadano ha iniciado sesión y no ha creado ningún reporte.
+WHEN: El ciudadano presiona " Seguimiento de Incidencias reportadas".
+THEN: La aplicación muestra un mensaje indicando que aún no tiene reportes registrados.
+Escenario 3: Ciudadano visualiza a detalle de una incidencia registrada
+GIVEN: El ciudadano hace click en "Seguimiento de incidencias"
+WHEN: El ciudadano presiona en "ver más detalles" sobre una incidencia específica en la lista de "Incidencias Registradas".
+THEN: La aplicación muestra todas las imágenes adjuntadas a la evidencia específica y la ubicación donde ocurrieron.</t>
+  </si>
+  <si>
+    <t>Escenario 1: Ciudadano consulta consejos sobre un tipo de residuo
+GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Educación Medioambiental".
+WHEN: El ciudadano selecciona "Residuos Orgánicos" en el combobox y confirma la consulta.
+THEN: La aplicación muestra al menos 2 recomendaciones que contribuyen al manejo correcto de ese tipo de residuo.
+Escenario 2: Ciudadano no selecciona ningún tipo de residuo
+GIVEN: El ciudadano ha iniciado sesión y se encuentra en "Educación Medioambiental".
+WHEN: El ciudadano intenta consultar sin seleccionar un tipo de residuo.
+THEN: El sistema muestra un mensaje solicitando que seleccione un tipo de residuo antes de continuar.
+Escenario 3: La IA no puede generar recomendaciones
+GIVEN: El ciudadano ha iniciado sesión, se encuentra en "Educación Medioambiental" y ha seleccionado un tipo de residuo.
+WHEN: El ciudadano confirma la consulta pero el servicio de IA no está disponible.
+THEN: El sistema muestra un mensaje indicando que no se pudieron generar las recomendaciones e invita al ciudadano a intentarlo más tarde.</t>
+  </si>
+  <si>
+    <t>Escenario 1: El sistema asigna puntos tras un registro exitoso
+GIVEN: El ciudadano ha completado y enviado correctamente una incidencia según HU014
+WHEN: El sistema confirma el registro de la incidencia
+THEN: El sistema asigna automáticamente los puntos correspondientes y notifica al ciudadano la cantidad de puntos ganados
+Escenario 2: Los puntos se reflejan inmediatamente en el perfil del ciudadano
+GIVEN:El ciudadano acaba de registrar una incidencia y el sistema le asignó puntos
+WHEN:El ciudadano accede a su perfil o sección "Mis puntos"
+THEN:El total de puntos mostrado incluye los puntos recién ganados
+Escenario 3:Incidencia duplicada no genera puntos adicionales
+GIVEN: El ciudadano intenta registrar una incidencia idéntica a una ya reportada por él
+WHEN: El sistema detecta la duplicidad y rechaza el registro
+THEN: No se asignan puntos adicionales y el sistema notifica que la incidencia ya fue registrada</t>
   </si>
 </sst>
 </file>
@@ -549,9 +550,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -587,6 +585,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -929,15 +930,18 @@
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="56.21875" customWidth="1"/>
+    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.77734375" customWidth="1"/>
+    <col min="13" max="13" width="53.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="11"/>
+      <c r="A3" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="10"/>
     </row>
     <row r="4" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
@@ -953,8 +957,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="268.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:4" ht="313.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="4" t="s">
@@ -967,8 +971,8 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="192.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="12"/>
+    <row r="6" spans="1:4" ht="260.39999999999998" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="11"/>
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
@@ -976,171 +980,171 @@
         <v>13</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="169.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="12"/>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="151.80000000000001" x14ac:dyDescent="0.3">
+      <c r="A7" s="11"/>
       <c r="B7" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="183" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="151.80000000000001" x14ac:dyDescent="0.3">
+      <c r="A8" s="7"/>
       <c r="B8" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="228.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
-        <v>32</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="343.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="228.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="343.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="13"/>
       <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>26</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="237" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="15"/>
+      <c r="A11" s="14"/>
       <c r="B11" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="200.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="364.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="7"/>
+      <c r="B13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="207" x14ac:dyDescent="0.3">
+      <c r="A14" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="201.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="5" t="s">
+      <c r="D14" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="331.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="17"/>
+      <c r="B15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="345" x14ac:dyDescent="0.3">
+      <c r="A16" s="17"/>
+      <c r="B16" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="304.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="14"/>
+      <c r="B17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="345.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="349.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="7"/>
+      <c r="B19" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>28</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="267.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="8"/>
-      <c r="B13" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="240.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="336" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="18"/>
-      <c r="B15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="364.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="18"/>
-      <c r="B16" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="331.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="15"/>
-      <c r="B17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="409.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="349.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>